<commit_message>
update formular in ratio sheet
</commit_message>
<xml_diff>
--- a/docs/templates/performance-ratios-template.xlsx
+++ b/docs/templates/performance-ratios-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\shidler\docs\templates\spreadsheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luongduyphuong/Documents/GitHub/Corporate-Finance-/docs/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_C2087B7F3B7CCEACD4328DE2D1E5418A185D2F1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759553C7-4324-BE4A-AFFA-587C8BA18CE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -1373,7 +1373,7 @@
     <xf numFmtId="49" fontId="18" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1381,7 +1381,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1682,10 +1682,32 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{DEAE66B9-B1B1-7C43-8685-CD563AF5FACE}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;2c165991-9a88-441c-be4a-ce298390d2af&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:C41"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -1693,39 +1715,39 @@
     <col min="4" max="4" width="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="8" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:3" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B4" s="51" t="s">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B4" s="45" t="s">
         <v>157</v>
       </c>
       <c r="C4" s="46"/>
     </row>
-    <row r="5" spans="2:3" ht="26" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="5" spans="2:3" ht="26" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="49" t="s">
         <v>158</v>
       </c>
       <c r="C5" s="46"/>
     </row>
-    <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="47" t="s">
         <v>159</v>
       </c>
       <c r="C6" s="46"/>
     </row>
-    <row r="7" spans="2:3" ht="4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" ht="4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
     </row>
-    <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="48" t="s">
         <v>160</v>
       </c>
       <c r="C9" s="46"/>
     </row>
-    <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
         <v>161</v>
       </c>
@@ -1733,7 +1755,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
         <v>163</v>
       </c>
@@ -1741,7 +1763,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
         <v>165</v>
       </c>
@@ -1749,7 +1771,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
         <v>167</v>
       </c>
@@ -1757,7 +1779,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="14" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
         <v>169</v>
       </c>
@@ -1765,7 +1787,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
         <v>171</v>
       </c>
@@ -1773,13 +1795,13 @@
         <v>172</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="48" t="s">
         <v>173</v>
       </c>
       <c r="C17" s="46"/>
     </row>
-    <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="5" t="s">
         <v>174</v>
       </c>
@@ -1787,7 +1809,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="6" t="s">
         <v>176</v>
       </c>
@@ -1795,7 +1817,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="8" t="s">
         <v>178</v>
       </c>
@@ -1803,7 +1825,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="9" t="s">
         <v>180</v>
       </c>
@@ -1811,7 +1833,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="10" t="s">
         <v>182</v>
       </c>
@@ -1819,13 +1841,13 @@
         <v>183</v>
       </c>
     </row>
-    <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="48" t="s">
         <v>184</v>
       </c>
       <c r="C24" s="46"/>
     </row>
-    <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="5" t="s">
         <v>185</v>
       </c>
@@ -1833,7 +1855,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
         <v>186</v>
       </c>
@@ -1841,7 +1863,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="27" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
         <v>188</v>
       </c>
@@ -1849,7 +1871,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="28" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="11" t="s">
         <v>190</v>
       </c>
@@ -1857,7 +1879,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="11" t="s">
         <v>192</v>
       </c>
@@ -1865,7 +1887,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="30" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="11" t="s">
         <v>194</v>
       </c>
@@ -1873,7 +1895,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="11" t="s">
         <v>196</v>
       </c>
@@ -1881,7 +1903,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="32" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="11" t="s">
         <v>198</v>
       </c>
@@ -1889,7 +1911,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="33" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="11" t="s">
         <v>200</v>
       </c>
@@ -1897,13 +1919,13 @@
         <v>201</v>
       </c>
     </row>
-    <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="48" t="s">
         <v>202</v>
       </c>
       <c r="C36" s="46"/>
     </row>
-    <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="12" t="s">
         <v>203</v>
       </c>
@@ -1911,7 +1933,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="38" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="12" t="s">
         <v>205</v>
       </c>
@@ -1919,7 +1941,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B41" s="50" t="s">
         <v>207</v>
       </c>
@@ -1943,7 +1965,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:H23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
@@ -1953,17 +1975,17 @@
     <col min="7" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:8" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="16" t="s">
         <v>210</v>
       </c>
@@ -1983,7 +2005,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="18" t="s">
         <v>214</v>
       </c>
@@ -1991,7 +2013,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
         <v>216</v>
       </c>
@@ -2003,7 +2025,7 @@
       <c r="G7" s="19"/>
       <c r="H7" s="19"/>
     </row>
-    <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
         <v>218</v>
       </c>
@@ -2015,7 +2037,7 @@
       <c r="G8" s="19"/>
       <c r="H8" s="19"/>
     </row>
-    <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
         <v>220</v>
       </c>
@@ -2027,7 +2049,7 @@
       <c r="G9" s="19"/>
       <c r="H9" s="19"/>
     </row>
-    <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="12" t="s">
         <v>222</v>
       </c>
@@ -2045,7 +2067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="20" t="s">
         <v>224</v>
       </c>
@@ -2058,14 +2080,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F12" s="12" t="s">
         <v>60</v>
       </c>
       <c r="G12" s="19"/>
       <c r="H12" s="19"/>
     </row>
-    <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="18" t="s">
         <v>225</v>
       </c>
@@ -2075,14 +2097,14 @@
       <c r="G13" s="19"/>
       <c r="H13" s="19"/>
     </row>
-    <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
         <v>227</v>
       </c>
       <c r="C14" s="19"/>
       <c r="D14" s="19"/>
     </row>
-    <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="12" t="s">
         <v>228</v>
       </c>
@@ -2100,7 +2122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
         <v>230</v>
       </c>
@@ -2113,12 +2135,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F17" s="18" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="18" t="s">
         <v>232</v>
       </c>
@@ -2128,7 +2150,7 @@
       <c r="G18" s="19"/>
       <c r="H18" s="19"/>
     </row>
-    <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="12" t="s">
         <v>234</v>
       </c>
@@ -2140,7 +2162,7 @@
       <c r="G19" s="19"/>
       <c r="H19" s="19"/>
     </row>
-    <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="12" t="s">
         <v>236</v>
       </c>
@@ -2158,8 +2180,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="23" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
         <v>238</v>
       </c>
@@ -2191,7 +2213,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:D19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
@@ -2199,17 +2221,17 @@
     <col min="4" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="23" t="s">
         <v>242</v>
       </c>
@@ -2220,7 +2242,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="12" t="s">
         <v>245</v>
       </c>
@@ -2229,7 +2251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
         <v>246</v>
       </c>
@@ -2239,7 +2261,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
         <v>247</v>
       </c>
@@ -2249,7 +2271,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
         <v>248</v>
       </c>
@@ -2259,7 +2281,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="20" t="s">
         <v>249</v>
       </c>
@@ -2272,7 +2294,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="12" t="s">
         <v>250</v>
       </c>
@@ -2282,7 +2304,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
         <v>251</v>
       </c>
@@ -2292,7 +2314,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="20" t="s">
         <v>252</v>
       </c>
@@ -2305,7 +2327,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
         <v>253</v>
       </c>
@@ -2315,7 +2337,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="5" t="s">
         <v>254</v>
       </c>
@@ -2328,12 +2350,12 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="18" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="12" t="s">
         <v>256</v>
       </c>
@@ -2343,7 +2365,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="20" t="s">
         <v>257</v>
       </c>
@@ -2364,7 +2386,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:D32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
@@ -2372,17 +2394,17 @@
     <col min="4" max="4" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="23" t="s">
         <v>242</v>
       </c>
@@ -2393,13 +2415,13 @@
         <v>259</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="18" t="s">
         <v>260</v>
       </c>
       <c r="D6" s="15"/>
     </row>
-    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
         <v>261</v>
       </c>
@@ -2411,7 +2433,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
         <v>263</v>
       </c>
@@ -2423,13 +2445,13 @@
         <v>262</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="28" t="s">
         <v>264</v>
       </c>
       <c r="D9" s="15"/>
     </row>
-    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="12" t="s">
         <v>265</v>
       </c>
@@ -2438,7 +2460,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="12" t="s">
         <v>267</v>
       </c>
@@ -2447,7 +2469,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
         <v>268</v>
       </c>
@@ -2456,7 +2478,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="12" t="s">
         <v>269</v>
       </c>
@@ -2465,7 +2487,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
         <v>270</v>
       </c>
@@ -2474,7 +2496,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="20" t="s">
         <v>271</v>
       </c>
@@ -2484,7 +2506,7 @@
       </c>
       <c r="D15" s="15"/>
     </row>
-    <row r="16" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="5" t="s">
         <v>272</v>
       </c>
@@ -2494,37 +2516,37 @@
       </c>
       <c r="D16" s="15"/>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D17" s="15"/>
     </row>
-    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="18" t="s">
         <v>273</v>
       </c>
       <c r="D18" s="15"/>
     </row>
-    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="12" t="s">
         <v>274</v>
       </c>
       <c r="C19" s="19"/>
       <c r="D19" s="15"/>
     </row>
-    <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="12" t="s">
         <v>275</v>
       </c>
       <c r="C20" s="19"/>
       <c r="D20" s="15"/>
     </row>
-    <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="12" t="s">
         <v>276</v>
       </c>
       <c r="C21" s="19"/>
       <c r="D21" s="15"/>
     </row>
-    <row r="22" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="5" t="s">
         <v>277</v>
       </c>
@@ -2534,51 +2556,51 @@
       </c>
       <c r="D22" s="15"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D23" s="15"/>
     </row>
-    <row r="24" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="18" t="s">
         <v>278</v>
       </c>
       <c r="D24" s="15"/>
     </row>
-    <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="12" t="s">
         <v>279</v>
       </c>
       <c r="C25" s="19"/>
       <c r="D25" s="15"/>
     </row>
-    <row r="26" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="12" t="s">
         <v>280</v>
       </c>
       <c r="C26" s="19"/>
       <c r="D26" s="15"/>
     </row>
-    <row r="27" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="12" t="s">
         <v>281</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="15"/>
     </row>
-    <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="12" t="s">
         <v>282</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="15"/>
     </row>
-    <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="12" t="s">
         <v>283</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="15"/>
     </row>
-    <row r="30" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="5" t="s">
         <v>284</v>
       </c>
@@ -2588,10 +2610,10 @@
       </c>
       <c r="D30" s="15"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D31" s="15"/>
     </row>
-    <row r="32" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="5" t="s">
         <v>285</v>
       </c>
@@ -2609,7 +2631,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B2:F76"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -2619,17 +2641,17 @@
     <col min="6" max="6" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="23" t="s">
         <v>2</v>
       </c>
@@ -2643,7 +2665,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="12" t="s">
         <v>6</v>
       </c>
@@ -2655,7 +2677,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
         <v>8</v>
       </c>
@@ -2670,7 +2692,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
         <v>11</v>
       </c>
@@ -2680,7 +2702,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
         <v>13</v>
       </c>
@@ -2690,7 +2712,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="12" t="s">
         <v>15</v>
       </c>
@@ -2702,7 +2724,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="12" t="s">
         <v>17</v>
       </c>
@@ -2714,7 +2736,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
         <v>19</v>
       </c>
@@ -2729,15 +2751,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="45" t="s">
+    <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="51" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="46"/>
       <c r="D14" s="46"/>
       <c r="E14" s="46"/>
     </row>
-    <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="12" t="s">
         <v>23</v>
       </c>
@@ -2752,7 +2774,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="12" t="s">
         <v>26</v>
       </c>
@@ -2767,7 +2789,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="12" t="s">
         <v>29</v>
       </c>
@@ -2782,7 +2804,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="12" t="s">
         <v>32</v>
       </c>
@@ -2797,7 +2819,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="12" t="s">
         <v>35</v>
       </c>
@@ -2812,15 +2834,15 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="45" t="s">
+    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="51" t="s">
         <v>38</v>
       </c>
       <c r="C21" s="46"/>
       <c r="D21" s="46"/>
       <c r="E21" s="46"/>
     </row>
-    <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="12" t="s">
         <v>39</v>
       </c>
@@ -2835,7 +2857,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="12" t="s">
         <v>42</v>
       </c>
@@ -2850,7 +2872,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="12" t="s">
         <v>45</v>
       </c>
@@ -2865,7 +2887,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="12" t="s">
         <v>48</v>
       </c>
@@ -2880,7 +2902,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="12" t="s">
         <v>51</v>
       </c>
@@ -2895,7 +2917,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="12" t="s">
         <v>54</v>
       </c>
@@ -2910,7 +2932,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="12" t="s">
         <v>57</v>
       </c>
@@ -2925,7 +2947,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="12" t="s">
         <v>60</v>
       </c>
@@ -2940,7 +2962,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="12" t="s">
         <v>63</v>
       </c>
@@ -2955,7 +2977,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="12" t="s">
         <v>66</v>
       </c>
@@ -2970,7 +2992,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="12" t="s">
         <v>69</v>
       </c>
@@ -2985,7 +3007,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="12" t="s">
         <v>72</v>
       </c>
@@ -3000,15 +3022,15 @@
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="45" t="s">
+    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="51" t="s">
         <v>75</v>
       </c>
       <c r="C35" s="46"/>
       <c r="D35" s="46"/>
       <c r="E35" s="46"/>
     </row>
-    <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="12" t="s">
         <v>76</v>
       </c>
@@ -3023,7 +3045,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="12" t="s">
         <v>79</v>
       </c>
@@ -3038,7 +3060,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="12" t="s">
         <v>82</v>
       </c>
@@ -3053,7 +3075,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="23" t="s">
         <v>85</v>
       </c>
@@ -3070,7 +3092,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="5" t="s">
         <v>89</v>
       </c>
@@ -3078,37 +3100,46 @@
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
     </row>
-    <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="C43" s="38"/>
+      <c r="C43" s="38">
+        <f>market_capitalization - currentYear_equity</f>
+        <v>0</v>
+      </c>
       <c r="D43" s="30" t="s">
         <v>91</v>
       </c>
       <c r="E43" s="30"/>
     </row>
-    <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B44" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="C44" s="39"/>
+      <c r="C44" s="39" t="e">
+        <f>market_capitalization / currentYear_equity</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D44" s="30" t="s">
         <v>93</v>
       </c>
       <c r="E44" s="30"/>
     </row>
-    <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="C45" s="38"/>
+      <c r="C45" s="38">
+        <f>currentYear_after_tax_operating_income-(cost_capital*startYear_total_capitalization)</f>
+        <v>0</v>
+      </c>
       <c r="D45" s="30" t="s">
         <v>95</v>
       </c>
       <c r="E45" s="30"/>
     </row>
-    <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B46" s="5" t="s">
         <v>96</v>
       </c>
@@ -3116,67 +3147,85 @@
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
     </row>
-    <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="C47" s="40"/>
+      <c r="C47" s="40" t="e">
+        <f>currentYear_after_tax_operating_income/startYear_total_assets</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D47" s="30" t="s">
         <v>98</v>
       </c>
       <c r="E47" s="30"/>
     </row>
-    <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="C48" s="40"/>
+      <c r="C48" s="40" t="e">
+        <f>currentYear_after_tax_operating_income/startYear_total_capitalization</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D48" s="30" t="s">
         <v>100</v>
       </c>
       <c r="E48" s="30"/>
     </row>
-    <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="C49" s="40"/>
+      <c r="C49" s="40" t="e">
+        <f>INC_net/startYear_equity</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D49" s="30" t="s">
         <v>102</v>
       </c>
       <c r="E49" s="30"/>
     </row>
-    <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="C50" s="40"/>
+      <c r="C50" s="40" t="e">
+        <f>currentYear_after_tax_operating_income/avg_total_assets</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D50" s="30" t="s">
         <v>104</v>
       </c>
       <c r="E50" s="30"/>
     </row>
-    <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C51" s="40"/>
+      <c r="C51" s="40" t="e">
+        <f>currentYear_after_tax_operating_income/avg_total_capitalization</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D51" s="30" t="s">
         <v>106</v>
       </c>
       <c r="E51" s="30"/>
     </row>
-    <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="C52" s="40"/>
+      <c r="C52" s="40" t="e">
+        <f>INC_net/avg_equity</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D52" s="30" t="s">
         <v>108</v>
       </c>
       <c r="E52" s="30"/>
     </row>
-    <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B53" s="5" t="s">
         <v>109</v>
       </c>
@@ -3184,11 +3233,14 @@
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
     </row>
-    <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B54" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="C54" s="39"/>
+      <c r="C54" s="39" t="e">
+        <f>INC_sales/startYear_total_assets</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D54" s="30" t="s">
         <v>111</v>
       </c>
@@ -3196,61 +3248,79 @@
         <v>112</v>
       </c>
     </row>
-    <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B55" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="C55" s="39"/>
+      <c r="C55" s="39" t="e">
+        <f>INC_sales/startYear_receivables</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D55" s="30" t="s">
         <v>114</v>
       </c>
       <c r="E55" s="30"/>
     </row>
-    <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B56" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="C56" s="41"/>
+      <c r="C56" s="41" t="e">
+        <f>startYear_receivables/currentYear_daily_sales_average</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D56" s="30" t="s">
         <v>116</v>
       </c>
       <c r="E56" s="30"/>
     </row>
-    <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="C57" s="39"/>
+      <c r="C57" s="39" t="e">
+        <f>INC_cost_goods_sold/startYear_inventory</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D57" s="30" t="s">
         <v>118</v>
       </c>
       <c r="E57" s="30"/>
     </row>
-    <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="C58" s="41"/>
+      <c r="C58" s="41" t="e">
+        <f>startYear_inventory/currentYear_cost_goods_sold_daily</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D58" s="30" t="s">
         <v>120</v>
       </c>
       <c r="E58" s="30"/>
     </row>
-    <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="C59" s="40"/>
+      <c r="C59" s="40" t="e">
+        <f>INC_net/INC_sales</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D59" s="30" t="s">
         <v>122</v>
       </c>
       <c r="E59" s="30"/>
     </row>
-    <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="C60" s="40"/>
+      <c r="C60" s="40" t="e">
+        <f>currentYear_after_tax_operating_income/INC_sales</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D60" s="30" t="s">
         <v>124</v>
       </c>
@@ -3258,7 +3328,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B61" s="5" t="s">
         <v>126</v>
       </c>
@@ -3266,61 +3336,79 @@
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
     </row>
-    <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B62" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="C62" s="40"/>
+      <c r="C62" s="40" t="e">
+        <f>currentYear_debt_long_term/(currentYear_debt_long_term+currentYear_equity)</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D62" s="30" t="s">
         <v>128</v>
       </c>
       <c r="E62" s="30"/>
     </row>
-    <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B63" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="C63" s="39"/>
+      <c r="C63" s="39" t="e">
+        <f>currentYear_debt_long_term/currentYear_equity</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D63" s="30" t="s">
         <v>130</v>
       </c>
       <c r="E63" s="30"/>
     </row>
-    <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B64" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="C64" s="40"/>
+      <c r="C64" s="40" t="e">
+        <f>currentYear_liabilities_total/currentYear_assets_total</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D64" s="30" t="s">
         <v>132</v>
       </c>
       <c r="E64" s="30"/>
     </row>
-    <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B65" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="C65" s="39"/>
+      <c r="C65" s="39" t="e">
+        <f>INC_ebit/INC_interest_expense</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D65" s="30" t="s">
         <v>134</v>
       </c>
       <c r="E65" s="30"/>
     </row>
-    <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B66" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="C66" s="39"/>
+      <c r="C66" s="39" t="e">
+        <f>(INC_ebit+INC_depreciation)/INC_interest_expense</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D66" s="30" t="s">
         <v>136</v>
       </c>
       <c r="E66" s="30"/>
     </row>
-    <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B67" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="C67" s="42"/>
+      <c r="C67" s="42" t="e">
+        <f>INC_net/currentYear_after_tax_operating_income</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D67" s="30" t="s">
         <v>138</v>
       </c>
@@ -3328,11 +3416,14 @@
         <v>139</v>
       </c>
     </row>
-    <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B68" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="C68" s="39"/>
+      <c r="C68" s="39" t="e">
+        <f>currentYear_assets_total/currentYear_equity</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D68" s="30" t="s">
         <v>141</v>
       </c>
@@ -3340,7 +3431,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B69" s="5" t="s">
         <v>143</v>
       </c>
@@ -3348,47 +3439,59 @@
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
     </row>
-    <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B70" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="C70" s="40"/>
+      <c r="C70" s="40" t="e">
+        <f>currentYear_working_capital_net/currentYear_assets_total</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D70" s="30" t="s">
         <v>145</v>
       </c>
       <c r="E70" s="30"/>
     </row>
-    <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B71" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="C71" s="39"/>
+      <c r="C71" s="39" t="e">
+        <f>currentYear_assets_current/currentYear_liabilities_current</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D71" s="30" t="s">
         <v>147</v>
       </c>
       <c r="E71" s="30"/>
     </row>
-    <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B72" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="C72" s="39"/>
+      <c r="C72" s="39" t="e">
+        <f>(currentYear_cash_marketable_securities+BAL_receivables_curr)/currentYear_liabilities_current</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D72" s="30" t="s">
         <v>149</v>
       </c>
       <c r="E72" s="30"/>
     </row>
-    <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B73" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="C73" s="39"/>
+      <c r="C73" s="39" t="e">
+        <f>currentYear_cash_marketable_securities/currentYear_liabilities_current</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D73" s="30" t="s">
         <v>151</v>
       </c>
       <c r="E73" s="30"/>
     </row>
-    <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B74" s="5" t="s">
         <v>152</v>
       </c>
@@ -3396,25 +3499,31 @@
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
     </row>
-    <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B75" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="C75" s="40"/>
+      <c r="C75" s="40" t="e">
+        <f>RATIO_asset_turnover*RATIO_operating_profit_margin</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D75" s="30" t="s">
         <v>154</v>
       </c>
       <c r="E75" s="30"/>
-      <c r="F75" s="44" t="str">
+      <c r="F75" s="44" t="e">
         <f>IF(OR(C75="",C47=""),"",IF(ROUND(C75,6)=ROUND(C47,6),"✓ matches direct ROA","✗ differs by "&amp;TEXT(ABS(C75-C47),"0.00%")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B76" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="C76" s="40"/>
+      <c r="C76" s="40" t="e">
+        <f>RATIO_leverage*RATIO_asset_turnover*RATIO_operating_profit_margin*RATIO_debt_burden</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="D76" s="30" t="s">
         <v>156</v>
       </c>
@@ -3433,19 +3542,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B2:C24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.90625" customWidth="1"/>
+    <col min="1" max="1" width="3.83203125" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:3" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="43" t="s">
         <v>287</v>
       </c>
@@ -3453,7 +3562,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="43" t="s">
         <v>289</v>
       </c>
@@ -3461,7 +3570,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="43" t="s">
         <v>291</v>
       </c>
@@ -3469,7 +3578,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" s="43" t="s">
         <v>293</v>
       </c>
@@ -3477,7 +3586,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="43" t="s">
         <v>295</v>
       </c>
@@ -3485,7 +3594,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="43" t="s">
         <v>296</v>
       </c>
@@ -3493,7 +3602,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="43" t="s">
         <v>298</v>
       </c>
@@ -3501,7 +3610,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="43" t="s">
         <v>299</v>
       </c>
@@ -3509,7 +3618,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="43" t="s">
         <v>301</v>
       </c>
@@ -3517,7 +3626,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" s="43" t="s">
         <v>303</v>
       </c>
@@ -3525,7 +3634,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14" s="43" t="s">
         <v>305</v>
       </c>
@@ -3533,7 +3642,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="43" t="s">
         <v>307</v>
       </c>
@@ -3541,7 +3650,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="43" t="s">
         <v>309</v>
       </c>
@@ -3549,7 +3658,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="43" t="s">
         <v>311</v>
       </c>
@@ -3557,7 +3666,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="43" t="s">
         <v>313</v>
       </c>
@@ -3565,7 +3674,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="43" t="s">
         <v>315</v>
       </c>
@@ -3573,12 +3682,12 @@
         <v>316</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" s="43" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="23" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="43" t="s">
         <v>318</v>
       </c>
@@ -3586,7 +3695,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="24" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="43" t="s">
         <v>320</v>
       </c>

</xml_diff>